<commit_message>
chore(mappa): aggiornamento automatico 2026-10-01
</commit_message>
<xml_diff>
--- a/Torino_2027.xlsx
+++ b/Torino_2027.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scarg\Dropbox\PNE Simone\Guide\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02F6DF98-634D-4955-A897-B9BD13D72BC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F9C4280-F075-4E68-B64A-8E152071FA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="665" xr2:uid="{65E54767-2A5A-433C-9949-276C98563996}"/>
   </bookViews>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2031" uniqueCount="917">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2031" uniqueCount="916">
   <si>
     <t>Recensore</t>
   </si>
@@ -2657,9 +2657,6 @@
   </si>
   <si>
     <t>Fernanda D'Arienzo</t>
-  </si>
-  <si>
-    <t>bloccato per Francesca Vasciaveo</t>
   </si>
   <si>
     <t>bloccato per Catia Gribaudo</t>
@@ -3800,15 +3797,15 @@
       </c>
       <c r="F4" s="4">
         <f>+AE6</f>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G4" s="4">
         <f>+AG6</f>
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H4" s="3">
         <f>+E4-G4</f>
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I4" s="39" t="s">
         <v>16</v>
@@ -3830,15 +3827,15 @@
       </c>
       <c r="F5" s="42">
         <f>+F3+F4</f>
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G5" s="42">
         <f>+G3+G4</f>
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H5" s="42">
         <f>+H3+H4</f>
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I5" s="43" t="s">
         <v>613</v>
@@ -3930,7 +3927,7 @@
       </c>
       <c r="AE6" s="1">
         <f t="shared" si="1"/>
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="AF6" s="1">
         <f t="shared" si="1"/>
@@ -3938,7 +3935,7 @@
       </c>
       <c r="AG6" s="1">
         <f t="shared" si="1"/>
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AH6" s="1">
         <f t="shared" si="1"/>
@@ -3999,7 +3996,7 @@
         <v>2</v>
       </c>
       <c r="Q7" s="45" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="R7" s="13"/>
       <c r="S7" s="13">
@@ -4113,7 +4110,7 @@
         <v>716</v>
       </c>
       <c r="N8" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O8" s="18">
         <v>1</v>
@@ -4367,7 +4364,7 @@
         <v>698</v>
       </c>
       <c r="N10" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O10" s="18">
         <v>1</v>
@@ -4469,7 +4466,7 @@
         <v>235</v>
       </c>
       <c r="F11" s="22" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="G11" s="22" t="s">
         <v>106</v>
@@ -4493,7 +4490,7 @@
         <v>678</v>
       </c>
       <c r="N11" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O11" s="18">
         <v>1</v>
@@ -4869,7 +4866,7 @@
         <v>194</v>
       </c>
       <c r="N14" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O14" s="18">
         <v>1</v>
@@ -4965,20 +4962,20 @@
         <v>2</v>
       </c>
       <c r="D15" s="28" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="E15" s="28" t="s">
         <v>276</v>
       </c>
       <c r="F15" s="28" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="G15" s="28"/>
       <c r="H15" s="28" t="s">
         <v>189</v>
       </c>
       <c r="I15" s="27" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="J15" s="27"/>
       <c r="K15" s="27" t="s">
@@ -5096,7 +5093,7 @@
         <v>189</v>
       </c>
       <c r="I16" s="29" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="J16" s="29">
         <v>1</v>
@@ -5233,7 +5230,7 @@
         <v>697</v>
       </c>
       <c r="N17" s="49" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="O17" s="18">
         <v>1</v>
@@ -5357,7 +5354,7 @@
         <v>809</v>
       </c>
       <c r="N18" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O18" s="18">
         <v>1</v>
@@ -5983,7 +5980,7 @@
         <v>245</v>
       </c>
       <c r="N23" s="49" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="O23" s="18">
         <v>1</v>
@@ -6109,7 +6106,7 @@
         <v>508</v>
       </c>
       <c r="N24" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O24" s="18">
         <v>1</v>
@@ -6235,7 +6232,7 @@
         <v>194</v>
       </c>
       <c r="N25" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O25" s="18">
         <v>1</v>
@@ -6361,7 +6358,7 @@
         <v>194</v>
       </c>
       <c r="N26" s="49" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="O26" s="18">
         <v>1</v>
@@ -6737,7 +6734,7 @@
         <v>699</v>
       </c>
       <c r="N29" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O29" s="18">
         <v>1</v>
@@ -6861,7 +6858,7 @@
         <v>790</v>
       </c>
       <c r="N30" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O30" s="18">
         <v>1</v>
@@ -6987,14 +6984,14 @@
         <v>700</v>
       </c>
       <c r="N31" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O31" s="18">
         <v>1</v>
       </c>
       <c r="P31" s="21"/>
       <c r="Q31" s="22" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="R31" s="5"/>
       <c r="S31" s="1">
@@ -7115,7 +7112,7 @@
         <v>245</v>
       </c>
       <c r="N32" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O32" s="18">
         <v>1</v>
@@ -7573,22 +7570,22 @@
         <v>5</v>
       </c>
       <c r="D36" s="22" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="E36" s="22" t="s">
         <v>233</v>
       </c>
       <c r="F36" s="22" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="G36" s="22" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="H36" s="22" t="s">
         <v>189</v>
       </c>
       <c r="I36" s="21" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="J36" s="21"/>
       <c r="K36" s="21" t="s">
@@ -7598,17 +7595,17 @@
         <v>55</v>
       </c>
       <c r="M36" s="57" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="N36" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O36" s="18">
         <v>1</v>
       </c>
       <c r="P36" s="21"/>
       <c r="Q36" s="22" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="R36" s="5"/>
       <c r="S36" s="1">
@@ -7729,7 +7726,7 @@
         <v>194</v>
       </c>
       <c r="N37" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O37" s="18">
         <v>1</v>
@@ -7983,7 +7980,7 @@
         <v>791</v>
       </c>
       <c r="N39" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O39" s="18">
         <v>1</v>
@@ -8231,7 +8228,7 @@
         <v>792</v>
       </c>
       <c r="N41" s="51" t="s">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="O41" s="19"/>
       <c r="P41" s="25"/>
@@ -8355,7 +8352,7 @@
         <v>692</v>
       </c>
       <c r="N42" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O42" s="18">
         <v>1</v>
@@ -9091,7 +9088,7 @@
         <v>511</v>
       </c>
       <c r="N48" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O48" s="18">
         <v>1</v>
@@ -9217,7 +9214,7 @@
         <v>676</v>
       </c>
       <c r="N49" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O49" s="18">
         <v>1</v>
@@ -9343,7 +9340,7 @@
         <v>300</v>
       </c>
       <c r="N50" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O50" s="18">
         <v>1</v>
@@ -9469,7 +9466,7 @@
         <v>194</v>
       </c>
       <c r="N51" s="49" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="O51" s="18">
         <v>1</v>
@@ -9595,7 +9592,7 @@
         <v>672</v>
       </c>
       <c r="N52" s="49" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="O52" s="18">
         <v>1</v>
@@ -9843,7 +9840,7 @@
         <v>300</v>
       </c>
       <c r="N54" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O54" s="18">
         <v>1</v>
@@ -9945,7 +9942,7 @@
         <v>234</v>
       </c>
       <c r="F55" s="22" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="G55" s="22" t="s">
         <v>488</v>
@@ -9969,7 +9966,7 @@
         <v>263</v>
       </c>
       <c r="N55" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O55" s="18">
         <v>1</v>
@@ -10098,7 +10095,7 @@
       <c r="O56" s="20"/>
       <c r="P56" s="23"/>
       <c r="Q56" s="24" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="R56" s="5"/>
       <c r="S56" s="1">
@@ -10189,13 +10186,13 @@
         <v>3</v>
       </c>
       <c r="D57" s="22" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="E57" s="22" t="s">
         <v>233</v>
       </c>
       <c r="F57" s="22" t="s">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="G57" s="22" t="s">
         <v>108</v>
@@ -10204,7 +10201,7 @@
         <v>189</v>
       </c>
       <c r="I57" s="21" t="s">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="J57" s="21"/>
       <c r="K57" s="21" t="s">
@@ -10679,51 +10676,53 @@
       <c r="AT60" s="5"/>
     </row>
     <row r="61" spans="1:46" s="6" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="25">
-        <v>0</v>
-      </c>
-      <c r="B61" s="25">
-        <v>1</v>
-      </c>
-      <c r="C61" s="25">
+      <c r="A61" s="21">
+        <v>0</v>
+      </c>
+      <c r="B61" s="21">
+        <v>1</v>
+      </c>
+      <c r="C61" s="21">
         <v>5</v>
       </c>
-      <c r="D61" s="26" t="s">
+      <c r="D61" s="22" t="s">
         <v>388</v>
       </c>
-      <c r="E61" s="26" t="s">
+      <c r="E61" s="22" t="s">
         <v>236</v>
       </c>
-      <c r="F61" s="26" t="s">
+      <c r="F61" s="22" t="s">
         <v>389</v>
       </c>
-      <c r="G61" s="26" t="s">
+      <c r="G61" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="H61" s="26" t="s">
+      <c r="H61" s="22" t="s">
         <v>189</v>
       </c>
-      <c r="I61" s="25" t="s">
+      <c r="I61" s="21" t="s">
         <v>390</v>
       </c>
-      <c r="J61" s="25">
+      <c r="J61" s="21">
         <v>5</v>
       </c>
-      <c r="K61" s="25" t="s">
+      <c r="K61" s="21" t="s">
         <v>296</v>
       </c>
-      <c r="L61" s="25" t="s">
+      <c r="L61" s="21" t="s">
         <v>303</v>
       </c>
-      <c r="M61" s="59" t="s">
+      <c r="M61" s="57" t="s">
         <v>673</v>
       </c>
-      <c r="N61" s="51" t="s">
-        <v>846</v>
-      </c>
-      <c r="O61" s="19"/>
-      <c r="P61" s="25"/>
-      <c r="Q61" s="26"/>
+      <c r="N61" s="49" t="s">
+        <v>852</v>
+      </c>
+      <c r="O61" s="18">
+        <v>1</v>
+      </c>
+      <c r="P61" s="21"/>
+      <c r="Q61" s="22"/>
       <c r="R61" s="5"/>
       <c r="S61" s="1">
         <f t="shared" si="23"/>
@@ -10772,7 +10771,7 @@
       </c>
       <c r="AE61" s="1">
         <f t="shared" si="34"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF61" s="1">
         <f t="shared" si="19"/>
@@ -10780,7 +10779,7 @@
       </c>
       <c r="AG61" s="1">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH61" s="1">
         <f t="shared" si="21"/>
@@ -11455,7 +11454,7 @@
         <v>675</v>
       </c>
       <c r="N67" s="49" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="O67" s="18">
         <v>1</v>
@@ -11581,7 +11580,7 @@
         <v>701</v>
       </c>
       <c r="N68" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O68" s="18">
         <v>1</v>
@@ -11707,7 +11706,7 @@
         <v>194</v>
       </c>
       <c r="N69" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O69" s="18">
         <v>1</v>
@@ -11803,13 +11802,13 @@
         <v>5</v>
       </c>
       <c r="D70" s="30" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="E70" s="30" t="s">
         <v>837</v>
       </c>
       <c r="F70" s="30" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="G70" s="30" t="s">
         <v>72</v>
@@ -11818,7 +11817,7 @@
         <v>189</v>
       </c>
       <c r="I70" s="29" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="J70" s="29">
         <v>4</v>
@@ -11830,7 +11829,7 @@
         <v>45</v>
       </c>
       <c r="M70" s="61" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="N70" s="53"/>
       <c r="O70" s="8"/>
@@ -11953,7 +11952,7 @@
         <v>814</v>
       </c>
       <c r="N71" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O71" s="18">
         <v>1</v>
@@ -12079,7 +12078,7 @@
         <v>710</v>
       </c>
       <c r="N72" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O72" s="18">
         <v>1</v>
@@ -12205,7 +12204,7 @@
         <v>511</v>
       </c>
       <c r="N73" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O73" s="18">
         <v>1</v>
@@ -12331,7 +12330,7 @@
         <v>511</v>
       </c>
       <c r="N74" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O74" s="18">
         <v>1</v>
@@ -12698,10 +12697,10 @@
         <v>70</v>
       </c>
       <c r="M77" s="57" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="N77" s="49" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="O77" s="18">
         <v>1</v>
@@ -13074,7 +13073,7 @@
       <c r="O80" s="8"/>
       <c r="P80" s="29"/>
       <c r="Q80" s="30" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="R80" s="5"/>
       <c r="S80" s="1">
@@ -13195,7 +13194,7 @@
         <v>506</v>
       </c>
       <c r="N81" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O81" s="18">
         <v>1</v>
@@ -13449,7 +13448,7 @@
         <v>247</v>
       </c>
       <c r="N83" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O83" s="18">
         <v>1</v>
@@ -13703,7 +13702,7 @@
         <v>709</v>
       </c>
       <c r="N85" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O85" s="18">
         <v>1</v>
@@ -13799,13 +13798,13 @@
         <v>6</v>
       </c>
       <c r="D86" s="22" t="s">
+        <v>874</v>
+      </c>
+      <c r="E86" s="22" t="s">
         <v>875</v>
       </c>
-      <c r="E86" s="22" t="s">
+      <c r="F86" s="22" t="s">
         <v>876</v>
-      </c>
-      <c r="F86" s="22" t="s">
-        <v>877</v>
       </c>
       <c r="G86" s="22" t="s">
         <v>88</v>
@@ -13814,7 +13813,7 @@
         <v>189</v>
       </c>
       <c r="I86" s="21" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="J86" s="21">
         <v>2</v>
@@ -13826,10 +13825,10 @@
         <v>45</v>
       </c>
       <c r="M86" s="57" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="N86" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O86" s="18">
         <v>1</v>
@@ -13952,7 +13951,7 @@
         <v>514</v>
       </c>
       <c r="N87" s="49" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="O87" s="18">
         <v>1</v>
@@ -14075,7 +14074,7 @@
         <v>514</v>
       </c>
       <c r="N88" s="49" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="O88" s="18">
         <v>1</v>
@@ -14201,7 +14200,7 @@
         <v>247</v>
       </c>
       <c r="N89" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O89" s="18">
         <v>1</v>
@@ -14297,20 +14296,20 @@
         <v>6</v>
       </c>
       <c r="D90" s="22" t="s">
+        <v>856</v>
+      </c>
+      <c r="E90" s="22" t="s">
         <v>857</v>
       </c>
-      <c r="E90" s="22" t="s">
+      <c r="F90" s="22" t="s">
         <v>858</v>
-      </c>
-      <c r="F90" s="22" t="s">
-        <v>859</v>
       </c>
       <c r="G90" s="22"/>
       <c r="H90" s="22" t="s">
         <v>189</v>
       </c>
       <c r="I90" s="21" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="J90" s="21"/>
       <c r="K90" s="21" t="s">
@@ -14447,7 +14446,7 @@
         <v>194</v>
       </c>
       <c r="N91" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O91" s="18">
         <v>1</v>
@@ -14573,7 +14572,7 @@
         <v>702</v>
       </c>
       <c r="N92" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O92" s="18">
         <v>1</v>
@@ -14821,7 +14820,7 @@
         <v>625</v>
       </c>
       <c r="N94" s="50" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O94" s="20">
         <v>1</v>
@@ -15212,7 +15211,7 @@
         <v>1</v>
       </c>
       <c r="Q97" s="22" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="R97" s="5"/>
       <c r="S97" s="1">
@@ -15333,7 +15332,7 @@
         <v>266</v>
       </c>
       <c r="N98" s="49" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="O98" s="18">
         <v>1</v>
@@ -15459,7 +15458,7 @@
         <v>266</v>
       </c>
       <c r="N99" s="49" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="O99" s="18">
         <v>1</v>
@@ -15585,7 +15584,7 @@
         <v>830</v>
       </c>
       <c r="N100" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O100" s="18">
         <v>1</v>
@@ -15711,7 +15710,7 @@
         <v>194</v>
       </c>
       <c r="N101" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O101" s="18">
         <v>1</v>
@@ -15959,7 +15958,7 @@
         <v>801</v>
       </c>
       <c r="N103" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O103" s="18">
         <v>1</v>
@@ -16085,7 +16084,7 @@
         <v>561</v>
       </c>
       <c r="N104" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O104" s="18">
         <v>1</v>
@@ -16211,7 +16210,7 @@
         <v>248</v>
       </c>
       <c r="N105" s="49" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="O105" s="18">
         <v>1</v>
@@ -16435,13 +16434,13 @@
         <v>1</v>
       </c>
       <c r="D107" s="22" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="E107" s="22" t="s">
         <v>69</v>
       </c>
       <c r="F107" s="22" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="G107" s="22" t="s">
         <v>88</v>
@@ -16450,7 +16449,7 @@
         <v>189</v>
       </c>
       <c r="I107" s="21" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="J107" s="21">
         <v>2</v>
@@ -16462,7 +16461,7 @@
         <v>5</v>
       </c>
       <c r="M107" s="57" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="N107" s="49" t="s">
         <v>845</v>
@@ -16474,7 +16473,7 @@
         <v>1</v>
       </c>
       <c r="Q107" s="22" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="R107" s="5"/>
       <c r="S107" s="1">
@@ -16604,7 +16603,7 @@
         <v>1</v>
       </c>
       <c r="Q108" s="22" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="R108" s="5"/>
       <c r="S108" s="1">
@@ -16695,7 +16694,7 @@
         <v>1</v>
       </c>
       <c r="D109" s="22" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="E109" s="22" t="s">
         <v>754</v>
@@ -17347,7 +17346,7 @@
         <v>192</v>
       </c>
       <c r="N114" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O114" s="18">
         <v>1</v>
@@ -18229,7 +18228,7 @@
         <v>704</v>
       </c>
       <c r="N121" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O121" s="18">
         <v>1</v>
@@ -18350,10 +18349,10 @@
         <v>30</v>
       </c>
       <c r="M122" s="57" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="N122" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O122" s="18">
         <v>1</v>
@@ -18607,7 +18606,7 @@
         <v>724</v>
       </c>
       <c r="N124" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O124" s="18">
         <v>1</v>
@@ -19075,7 +19074,7 @@
         <v>380</v>
       </c>
       <c r="F128" s="30" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="G128" s="30" t="s">
         <v>203</v>
@@ -19557,18 +19556,18 @@
         <v>2</v>
       </c>
       <c r="D132" s="22" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="E132" s="22"/>
       <c r="F132" s="22" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="G132" s="22"/>
       <c r="H132" s="22" t="s">
         <v>189</v>
       </c>
       <c r="I132" s="21" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="J132" s="21"/>
       <c r="K132" s="21" t="s">
@@ -19578,7 +19577,7 @@
         <v>22</v>
       </c>
       <c r="M132" s="57" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="N132" s="49" t="s">
         <v>845</v>
@@ -19837,7 +19836,7 @@
         <v>454</v>
       </c>
       <c r="N134" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O134" s="18">
         <v>1</v>
@@ -20085,7 +20084,7 @@
         <v>665</v>
       </c>
       <c r="N136" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O136" s="18">
         <v>1</v>
@@ -20693,13 +20692,13 @@
         <v>3</v>
       </c>
       <c r="D141" s="22" t="s">
+        <v>867</v>
+      </c>
+      <c r="E141" s="22" t="s">
+        <v>866</v>
+      </c>
+      <c r="F141" s="22" t="s">
         <v>868</v>
-      </c>
-      <c r="E141" s="22" t="s">
-        <v>867</v>
-      </c>
-      <c r="F141" s="22" t="s">
-        <v>869</v>
       </c>
       <c r="G141" s="22" t="s">
         <v>136</v>
@@ -20823,7 +20822,7 @@
         <v>633</v>
       </c>
       <c r="F142" s="22" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="G142" s="22" t="s">
         <v>83</v>
@@ -20856,7 +20855,7 @@
         <v>1</v>
       </c>
       <c r="Q142" s="22" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="R142" s="5"/>
       <c r="S142" s="1">
@@ -21351,7 +21350,7 @@
         <v>666</v>
       </c>
       <c r="N146" s="49" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="O146" s="18">
         <v>1</v>
@@ -21599,7 +21598,7 @@
         <v>620</v>
       </c>
       <c r="N148" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O148" s="18">
         <v>1</v>
@@ -21725,7 +21724,7 @@
         <v>512</v>
       </c>
       <c r="N149" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O149" s="18">
         <v>1</v>
@@ -22226,7 +22225,7 @@
         <v>667</v>
       </c>
       <c r="N153" s="50" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="O153" s="20"/>
       <c r="P153" s="23"/>
@@ -22588,7 +22587,7 @@
         <v>814</v>
       </c>
       <c r="N156" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O156" s="18">
         <v>1</v>
@@ -22714,7 +22713,7 @@
         <v>727</v>
       </c>
       <c r="N157" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O157" s="18">
         <v>1</v>
@@ -22962,7 +22961,7 @@
         <v>840</v>
       </c>
       <c r="N159" s="49" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="O159" s="18">
         <v>1</v>
@@ -23084,7 +23083,7 @@
         <v>825</v>
       </c>
       <c r="N160" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O160" s="18">
         <v>1</v>
@@ -23210,7 +23209,7 @@
         <v>459</v>
       </c>
       <c r="N161" s="49" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="O161" s="18">
         <v>1</v>
@@ -23330,10 +23329,10 @@
         <v>45</v>
       </c>
       <c r="M162" s="59" t="s">
+        <v>914</v>
+      </c>
+      <c r="N162" s="51" t="s">
         <v>915</v>
-      </c>
-      <c r="N162" s="51" t="s">
-        <v>916</v>
       </c>
       <c r="O162" s="19"/>
       <c r="P162" s="25"/>
@@ -23701,7 +23700,7 @@
         <v>742</v>
       </c>
       <c r="N165" s="49" t="s">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="O165" s="18">
         <v>1</v>
@@ -24053,7 +24052,7 @@
         <v>87</v>
       </c>
       <c r="F168" s="30" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="G168" s="30" t="s">
         <v>99</v>
@@ -24303,7 +24302,7 @@
         <v>38</v>
       </c>
       <c r="F170" s="22" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="G170" s="22" t="s">
         <v>82</v>
@@ -24559,7 +24558,7 @@
         <v>38</v>
       </c>
       <c r="F172" s="22" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="G172" s="22" t="s">
         <v>756</v>
@@ -24839,7 +24838,7 @@
         <v>195</v>
       </c>
       <c r="N174" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O174" s="18">
         <v>1</v>
@@ -24950,7 +24949,7 @@
         <v>189</v>
       </c>
       <c r="I175" s="21" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="J175" s="21">
         <v>99</v>
@@ -24965,7 +24964,7 @@
         <v>195</v>
       </c>
       <c r="N175" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O175" s="18">
         <v>1</v>
@@ -25076,7 +25075,7 @@
         <v>189</v>
       </c>
       <c r="I176" s="21" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="J176" s="21"/>
       <c r="K176" s="21" t="s">
@@ -25089,7 +25088,7 @@
         <v>195</v>
       </c>
       <c r="N176" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O176" s="18">
         <v>1</v>
@@ -26084,7 +26083,7 @@
         <v>195</v>
       </c>
       <c r="N184" s="51" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="O184" s="19"/>
       <c r="P184" s="25"/>
@@ -27684,7 +27683,7 @@
         <v>55</v>
       </c>
       <c r="F197" s="22" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="G197" s="22" t="s">
         <v>72</v>
@@ -27693,7 +27692,7 @@
         <v>189</v>
       </c>
       <c r="I197" s="21" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="J197" s="21">
         <v>4</v>
@@ -28458,7 +28457,7 @@
         <v>195</v>
       </c>
       <c r="N203" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O203" s="18">
         <v>1</v>
@@ -28584,7 +28583,7 @@
         <v>195</v>
       </c>
       <c r="N204" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O204" s="18">
         <v>1</v>
@@ -28680,7 +28679,7 @@
         <v>7</v>
       </c>
       <c r="D205" s="22" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="E205" s="22" t="s">
         <v>38</v>
@@ -28808,7 +28807,7 @@
         <v>7</v>
       </c>
       <c r="D206" s="22" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="E206" s="22" t="s">
         <v>38</v>
@@ -28966,7 +28965,7 @@
         <v>195</v>
       </c>
       <c r="N207" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O207" s="18">
         <v>1</v>
@@ -29092,7 +29091,7 @@
         <v>195</v>
       </c>
       <c r="N208" s="49" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="O208" s="18">
         <v>1</v>
@@ -30075,7 +30074,7 @@
         <v>55</v>
       </c>
       <c r="F216" s="22" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="G216" s="22" t="s">
         <v>144</v>
@@ -30224,7 +30223,7 @@
         <v>310</v>
       </c>
       <c r="N217" s="51" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="O217" s="19"/>
       <c r="P217" s="25"/>

</xml_diff>